<commit_message>
Atualização automática: 2026-08-03 15:47
</commit_message>
<xml_diff>
--- a/data/base_formatada/Base.xlsx
+++ b/data/base_formatada/Base.xlsx
@@ -5965,7 +5965,7 @@
     <t>Shofia Gomes</t>
   </si>
   <si>
-    <t>Denis Reis</t>
+    <t>Gustavo Tonan</t>
   </si>
   <si>
     <t>Priscila Volpe</t>
@@ -29439,7 +29439,7 @@
         <v>1854</v>
       </c>
       <c r="E469" t="s">
-        <v>1871</v>
+        <v>1873</v>
       </c>
       <c r="F469" t="s">
         <v>1888</v>
@@ -29489,7 +29489,7 @@
         <v>1854</v>
       </c>
       <c r="E470" t="s">
-        <v>1871</v>
+        <v>1873</v>
       </c>
       <c r="F470" t="s">
         <v>1888</v>
@@ -29539,7 +29539,7 @@
         <v>1854</v>
       </c>
       <c r="E471" t="s">
-        <v>1871</v>
+        <v>1873</v>
       </c>
       <c r="F471" t="s">
         <v>1888</v>
@@ -29839,7 +29839,7 @@
         <v>1854</v>
       </c>
       <c r="E477" t="s">
-        <v>1871</v>
+        <v>1873</v>
       </c>
       <c r="F477" t="s">
         <v>1886</v>

</xml_diff>

<commit_message>
Atualização automática: 2026-08-05 17:51
</commit_message>
<xml_diff>
--- a/data/base_formatada/Base.xlsx
+++ b/data/base_formatada/Base.xlsx
@@ -1597,7 +1597,7 @@
     <t>DINIZ DISTRIBUIDORA DE PRODUTOS ALIMENTICIOS LTDA</t>
   </si>
   <si>
-    <t>ARMERINA IMÓVEIS EIRELI</t>
+    <t>ARMERINA IMÓVEIS LTDA</t>
   </si>
   <si>
     <t>ÁGUA LIMPA DISTRIBUIDORA DE HORTIFRUTI, ALIMENTOS E SERVIÇOS DE TRANSPORTES LTDA.</t>
@@ -57717,7 +57717,7 @@
         <v>1852</v>
       </c>
       <c r="E1048" t="s">
-        <v>1884</v>
+        <v>1873</v>
       </c>
       <c r="F1048" t="s">
         <v>1887</v>

</xml_diff>

<commit_message>
Atualização automática: 2026-08-07 09:28
</commit_message>
<xml_diff>
--- a/data/base_formatada/Base.xlsx
+++ b/data/base_formatada/Base.xlsx
@@ -16514,7 +16514,7 @@
         <v>1403</v>
       </c>
       <c r="D206" t="s">
-        <v>1854</v>
+        <v>1861</v>
       </c>
       <c r="E206" t="s">
         <v>1874</v>
@@ -16564,7 +16564,7 @@
         <v>1403</v>
       </c>
       <c r="D207" t="s">
-        <v>1854</v>
+        <v>1861</v>
       </c>
       <c r="E207" t="s">
         <v>1874</v>
@@ -32406,7 +32406,7 @@
         <v>1498</v>
       </c>
       <c r="D529" t="s">
-        <v>1853</v>
+        <v>1854</v>
       </c>
       <c r="E529" t="s">
         <v>1874</v>

</xml_diff>

<commit_message>
Atualização automática: 2026-08-10 11:07
</commit_message>
<xml_diff>
--- a/data/base_formatada/Base.xlsx
+++ b/data/base_formatada/Base.xlsx
@@ -5845,46 +5845,46 @@
     <t>Leidiane Paulino</t>
   </si>
   <si>
+    <t>Maria Eduarda</t>
+  </si>
+  <si>
+    <t>Walace Gonçalves</t>
+  </si>
+  <si>
+    <t>Veronica Barbosa</t>
+  </si>
+  <si>
+    <t>Nata Trindade</t>
+  </si>
+  <si>
+    <t>Karen Corazza</t>
+  </si>
+  <si>
+    <t>Danielle Silva</t>
+  </si>
+  <si>
+    <t>Rangel Rocha</t>
+  </si>
+  <si>
+    <t>Pamella Sersosimo</t>
+  </si>
+  <si>
+    <t>Kellem Freitas</t>
+  </si>
+  <si>
+    <t>Simone Soares</t>
+  </si>
+  <si>
+    <t>Suzana Silva</t>
+  </si>
+  <si>
+    <t>Jeniffer Cristina</t>
+  </si>
+  <si>
+    <t>Luis Junior</t>
+  </si>
+  <si>
     <t>Vitoria Silva</t>
-  </si>
-  <si>
-    <t>Maria Eduarda</t>
-  </si>
-  <si>
-    <t>Walace Gonçalves</t>
-  </si>
-  <si>
-    <t>Veronica Barbosa</t>
-  </si>
-  <si>
-    <t>Nata Trindade</t>
-  </si>
-  <si>
-    <t>Karen Corazza</t>
-  </si>
-  <si>
-    <t>Danielle Silva</t>
-  </si>
-  <si>
-    <t>Rangel Rocha</t>
-  </si>
-  <si>
-    <t>Pamella Sersosimo</t>
-  </si>
-  <si>
-    <t>Kellem Freitas</t>
-  </si>
-  <si>
-    <t>Simone Soares</t>
-  </si>
-  <si>
-    <t>Suzana Silva</t>
-  </si>
-  <si>
-    <t>Jeniffer Cristina</t>
-  </si>
-  <si>
-    <t>Luis Junior</t>
   </si>
   <si>
     <t>Bianca Silva</t>
@@ -24977,7 +24977,7 @@
         <v>2018</v>
       </c>
       <c r="N377" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O377" t="s">
         <v>2029</v>
@@ -25700,7 +25700,7 @@
         <v>2018</v>
       </c>
       <c r="N392" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O392" t="s">
         <v>2031</v>
@@ -25847,7 +25847,7 @@
         <v>2018</v>
       </c>
       <c r="N395" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O395" t="s">
         <v>2031</v>
@@ -25923,7 +25923,7 @@
         <v>1893</v>
       </c>
       <c r="H397" t="s">
-        <v>1943</v>
+        <v>1941</v>
       </c>
       <c r="I397" t="s">
         <v>1995</v>
@@ -25941,7 +25941,7 @@
         <v>2018</v>
       </c>
       <c r="N397" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O397" t="s">
         <v>2029</v>
@@ -26217,7 +26217,7 @@
         <v>1893</v>
       </c>
       <c r="H403" t="s">
-        <v>1944</v>
+        <v>1943</v>
       </c>
       <c r="I403" t="s">
         <v>1996</v>
@@ -26282,7 +26282,7 @@
         <v>2018</v>
       </c>
       <c r="N404" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O404" t="s">
         <v>2031</v>
@@ -26458,7 +26458,7 @@
         <v>1893</v>
       </c>
       <c r="H408" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="I408" t="s">
         <v>1995</v>
@@ -26476,7 +26476,7 @@
         <v>2018</v>
       </c>
       <c r="N408" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O408" t="s">
         <v>2031</v>
@@ -26502,7 +26502,7 @@
         <v>1893</v>
       </c>
       <c r="H409" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="I409" t="s">
         <v>1995</v>
@@ -26520,7 +26520,7 @@
         <v>2018</v>
       </c>
       <c r="N409" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O409" t="s">
         <v>2031</v>
@@ -26552,7 +26552,7 @@
         <v>1893</v>
       </c>
       <c r="H410" t="s">
-        <v>1946</v>
+        <v>1945</v>
       </c>
       <c r="I410" t="s">
         <v>1995</v>
@@ -26570,7 +26570,7 @@
         <v>2016</v>
       </c>
       <c r="N410" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O410" t="s">
         <v>2029</v>
@@ -26602,7 +26602,7 @@
         <v>1893</v>
       </c>
       <c r="H411" t="s">
-        <v>1946</v>
+        <v>1945</v>
       </c>
       <c r="I411" t="s">
         <v>1995</v>
@@ -26620,7 +26620,7 @@
         <v>2018</v>
       </c>
       <c r="N411" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O411" t="s">
         <v>2031</v>
@@ -26652,7 +26652,7 @@
         <v>1893</v>
       </c>
       <c r="H412" t="s">
-        <v>1946</v>
+        <v>1945</v>
       </c>
       <c r="I412" t="s">
         <v>1995</v>
@@ -26670,7 +26670,7 @@
         <v>2018</v>
       </c>
       <c r="N412" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O412" t="s">
         <v>2031</v>
@@ -26952,7 +26952,7 @@
         <v>1893</v>
       </c>
       <c r="H418" t="s">
-        <v>1947</v>
+        <v>1946</v>
       </c>
       <c r="I418" t="s">
         <v>1992</v>
@@ -27343,7 +27343,7 @@
         <v>1893</v>
       </c>
       <c r="H426" t="s">
-        <v>1948</v>
+        <v>1947</v>
       </c>
       <c r="I426" t="s">
         <v>1997</v>
@@ -27390,7 +27390,7 @@
         <v>1893</v>
       </c>
       <c r="H427" t="s">
-        <v>1948</v>
+        <v>1947</v>
       </c>
       <c r="I427" t="s">
         <v>1997</v>
@@ -27437,7 +27437,7 @@
         <v>1893</v>
       </c>
       <c r="H428" t="s">
-        <v>1948</v>
+        <v>1947</v>
       </c>
       <c r="I428" t="s">
         <v>1997</v>
@@ -27484,7 +27484,7 @@
         <v>1893</v>
       </c>
       <c r="H429" t="s">
-        <v>1948</v>
+        <v>1947</v>
       </c>
       <c r="I429" t="s">
         <v>1997</v>
@@ -27531,7 +27531,7 @@
         <v>1893</v>
       </c>
       <c r="H430" t="s">
-        <v>1948</v>
+        <v>1947</v>
       </c>
       <c r="I430" t="s">
         <v>1997</v>
@@ -27622,7 +27622,7 @@
         <v>1893</v>
       </c>
       <c r="H432" t="s">
-        <v>1949</v>
+        <v>1948</v>
       </c>
       <c r="I432" t="s">
         <v>1989</v>
@@ -28063,7 +28063,7 @@
         <v>1893</v>
       </c>
       <c r="H441" t="s">
-        <v>1950</v>
+        <v>1949</v>
       </c>
       <c r="I441" t="s">
         <v>1995</v>
@@ -28081,7 +28081,7 @@
         <v>2018</v>
       </c>
       <c r="N441" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O441" t="s">
         <v>2031</v>
@@ -28113,7 +28113,7 @@
         <v>1893</v>
       </c>
       <c r="H442" t="s">
-        <v>1950</v>
+        <v>1949</v>
       </c>
       <c r="I442" t="s">
         <v>1995</v>
@@ -28131,7 +28131,7 @@
         <v>2019</v>
       </c>
       <c r="N442" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O442" t="s">
         <v>2029</v>
@@ -28163,7 +28163,7 @@
         <v>1893</v>
       </c>
       <c r="H443" t="s">
-        <v>1950</v>
+        <v>1949</v>
       </c>
       <c r="I443" t="s">
         <v>1995</v>
@@ -28181,7 +28181,7 @@
         <v>2018</v>
       </c>
       <c r="N443" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O443" t="s">
         <v>2031</v>
@@ -28213,7 +28213,7 @@
         <v>1893</v>
       </c>
       <c r="H444" t="s">
-        <v>1950</v>
+        <v>1949</v>
       </c>
       <c r="I444" t="s">
         <v>1995</v>
@@ -28231,7 +28231,7 @@
         <v>2018</v>
       </c>
       <c r="N444" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O444" t="s">
         <v>2031</v>
@@ -28263,7 +28263,7 @@
         <v>1893</v>
       </c>
       <c r="H445" t="s">
-        <v>1951</v>
+        <v>1950</v>
       </c>
       <c r="I445" t="s">
         <v>1996</v>
@@ -28310,7 +28310,7 @@
         <v>1893</v>
       </c>
       <c r="H446" t="s">
-        <v>1951</v>
+        <v>1950</v>
       </c>
       <c r="I446" t="s">
         <v>1996</v>
@@ -28357,7 +28357,7 @@
         <v>1893</v>
       </c>
       <c r="H447" t="s">
-        <v>1952</v>
+        <v>1951</v>
       </c>
       <c r="I447" t="s">
         <v>1995</v>
@@ -28375,7 +28375,7 @@
         <v>2018</v>
       </c>
       <c r="N447" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O447" t="s">
         <v>2031</v>
@@ -28407,7 +28407,7 @@
         <v>1893</v>
       </c>
       <c r="H448" t="s">
-        <v>1952</v>
+        <v>1951</v>
       </c>
       <c r="I448" t="s">
         <v>1995</v>
@@ -28425,7 +28425,7 @@
         <v>2018</v>
       </c>
       <c r="N448" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O448" t="s">
         <v>2031</v>
@@ -28457,7 +28457,7 @@
         <v>1893</v>
       </c>
       <c r="H449" t="s">
-        <v>1952</v>
+        <v>1951</v>
       </c>
       <c r="I449" t="s">
         <v>1995</v>
@@ -28475,7 +28475,7 @@
         <v>2018</v>
       </c>
       <c r="N449" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O449" t="s">
         <v>2031</v>
@@ -28507,7 +28507,7 @@
         <v>1893</v>
       </c>
       <c r="H450" t="s">
-        <v>1952</v>
+        <v>1951</v>
       </c>
       <c r="I450" t="s">
         <v>1995</v>
@@ -28525,7 +28525,7 @@
         <v>2018</v>
       </c>
       <c r="N450" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O450" t="s">
         <v>2031</v>
@@ -28557,7 +28557,7 @@
         <v>1893</v>
       </c>
       <c r="H451" t="s">
-        <v>1952</v>
+        <v>1951</v>
       </c>
       <c r="I451" t="s">
         <v>1995</v>
@@ -28575,7 +28575,7 @@
         <v>2018</v>
       </c>
       <c r="N451" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O451" t="s">
         <v>2031</v>
@@ -28607,7 +28607,7 @@
         <v>1893</v>
       </c>
       <c r="H452" t="s">
-        <v>1952</v>
+        <v>1951</v>
       </c>
       <c r="I452" t="s">
         <v>1995</v>
@@ -28625,7 +28625,7 @@
         <v>2018</v>
       </c>
       <c r="N452" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O452" t="s">
         <v>2031</v>
@@ -28704,7 +28704,7 @@
         <v>1893</v>
       </c>
       <c r="H454" t="s">
-        <v>1953</v>
+        <v>1952</v>
       </c>
       <c r="I454" t="s">
         <v>1995</v>
@@ -28722,7 +28722,7 @@
         <v>2018</v>
       </c>
       <c r="N454" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O454" t="s">
         <v>2031</v>
@@ -28754,7 +28754,7 @@
         <v>1893</v>
       </c>
       <c r="H455" t="s">
-        <v>1954</v>
+        <v>1953</v>
       </c>
       <c r="I455" t="s">
         <v>1995</v>
@@ -28772,7 +28772,7 @@
         <v>2018</v>
       </c>
       <c r="N455" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O455" t="s">
         <v>2029</v>
@@ -29001,7 +29001,7 @@
         <v>1893</v>
       </c>
       <c r="H460" t="s">
-        <v>1943</v>
+        <v>1941</v>
       </c>
       <c r="I460" t="s">
         <v>1995</v>
@@ -29019,7 +29019,7 @@
         <v>2016</v>
       </c>
       <c r="N460" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O460" t="s">
         <v>2029</v>
@@ -29051,7 +29051,7 @@
         <v>1893</v>
       </c>
       <c r="H461" t="s">
-        <v>1943</v>
+        <v>1941</v>
       </c>
       <c r="I461" t="s">
         <v>1995</v>
@@ -29069,7 +29069,7 @@
         <v>2018</v>
       </c>
       <c r="N461" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O461" t="s">
         <v>2031</v>
@@ -29101,7 +29101,7 @@
         <v>1893</v>
       </c>
       <c r="H462" t="s">
-        <v>1943</v>
+        <v>1941</v>
       </c>
       <c r="I462" t="s">
         <v>1995</v>
@@ -29119,7 +29119,7 @@
         <v>2018</v>
       </c>
       <c r="N462" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O462" t="s">
         <v>2029</v>
@@ -29151,7 +29151,7 @@
         <v>1893</v>
       </c>
       <c r="H463" t="s">
-        <v>1952</v>
+        <v>1951</v>
       </c>
       <c r="I463" t="s">
         <v>1995</v>
@@ -29169,7 +29169,7 @@
         <v>2018</v>
       </c>
       <c r="N463" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O463" t="s">
         <v>2031</v>
@@ -29769,7 +29769,7 @@
         <v>2018</v>
       </c>
       <c r="N475" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O475" t="s">
         <v>2031</v>
@@ -29801,7 +29801,7 @@
         <v>1893</v>
       </c>
       <c r="H476" t="s">
-        <v>1952</v>
+        <v>1951</v>
       </c>
       <c r="I476" t="s">
         <v>1995</v>
@@ -29819,7 +29819,7 @@
         <v>2018</v>
       </c>
       <c r="N476" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O476" t="s">
         <v>2031</v>
@@ -30101,7 +30101,7 @@
         <v>1893</v>
       </c>
       <c r="H482" t="s">
-        <v>1955</v>
+        <v>1954</v>
       </c>
       <c r="I482" t="s">
         <v>1995</v>
@@ -30119,7 +30119,7 @@
         <v>2018</v>
       </c>
       <c r="N482" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O482" t="s">
         <v>2031</v>
@@ -30592,7 +30592,7 @@
         <v>1893</v>
       </c>
       <c r="H492" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="I492" t="s">
         <v>1995</v>
@@ -30610,7 +30610,7 @@
         <v>2018</v>
       </c>
       <c r="N492" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O492" t="s">
         <v>2031</v>
@@ -30739,7 +30739,7 @@
         <v>1893</v>
       </c>
       <c r="H495" t="s">
-        <v>1956</v>
+        <v>1955</v>
       </c>
       <c r="I495" t="s">
         <v>1995</v>
@@ -30757,7 +30757,7 @@
         <v>2020</v>
       </c>
       <c r="N495" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O495" t="s">
         <v>2030</v>
@@ -30857,7 +30857,7 @@
         <v>2018</v>
       </c>
       <c r="N497" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O497" t="s">
         <v>2031</v>
@@ -30907,7 +30907,7 @@
         <v>2018</v>
       </c>
       <c r="N498" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O498" t="s">
         <v>2031</v>
@@ -31039,7 +31039,7 @@
         <v>1893</v>
       </c>
       <c r="H501" t="s">
-        <v>1943</v>
+        <v>1956</v>
       </c>
       <c r="I501" t="s">
         <v>1995</v>
@@ -31057,7 +31057,7 @@
         <v>2018</v>
       </c>
       <c r="N501" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O501" t="s">
         <v>2031</v>
@@ -31289,7 +31289,7 @@
         <v>1893</v>
       </c>
       <c r="H506" t="s">
-        <v>1946</v>
+        <v>1945</v>
       </c>
       <c r="I506" t="s">
         <v>1995</v>
@@ -31307,7 +31307,7 @@
         <v>2016</v>
       </c>
       <c r="N506" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O506" t="s">
         <v>2029</v>
@@ -31486,7 +31486,7 @@
         <v>1893</v>
       </c>
       <c r="H510" t="s">
-        <v>1947</v>
+        <v>1946</v>
       </c>
       <c r="I510" t="s">
         <v>1992</v>
@@ -31804,7 +31804,7 @@
         <v>2018</v>
       </c>
       <c r="N516" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O516" t="s">
         <v>2031</v>
@@ -31986,7 +31986,7 @@
         <v>1893</v>
       </c>
       <c r="H520" t="s">
-        <v>1946</v>
+        <v>1945</v>
       </c>
       <c r="I520" t="s">
         <v>1995</v>
@@ -32004,7 +32004,7 @@
         <v>2018</v>
       </c>
       <c r="N520" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O520" t="s">
         <v>2031</v>
@@ -32036,7 +32036,7 @@
         <v>1893</v>
       </c>
       <c r="H521" t="s">
-        <v>1948</v>
+        <v>1947</v>
       </c>
       <c r="I521" t="s">
         <v>1997</v>
@@ -32083,7 +32083,7 @@
         <v>1893</v>
       </c>
       <c r="H522" t="s">
-        <v>1948</v>
+        <v>1947</v>
       </c>
       <c r="I522" t="s">
         <v>1997</v>
@@ -32130,7 +32130,7 @@
         <v>1893</v>
       </c>
       <c r="H523" t="s">
-        <v>1948</v>
+        <v>1947</v>
       </c>
       <c r="I523" t="s">
         <v>1997</v>
@@ -32177,7 +32177,7 @@
         <v>1893</v>
       </c>
       <c r="H524" t="s">
-        <v>1948</v>
+        <v>1947</v>
       </c>
       <c r="I524" t="s">
         <v>1997</v>
@@ -32224,7 +32224,7 @@
         <v>1893</v>
       </c>
       <c r="H525" t="s">
-        <v>1948</v>
+        <v>1947</v>
       </c>
       <c r="I525" t="s">
         <v>1997</v>
@@ -32271,7 +32271,7 @@
         <v>1893</v>
       </c>
       <c r="H526" t="s">
-        <v>1948</v>
+        <v>1947</v>
       </c>
       <c r="I526" t="s">
         <v>1997</v>
@@ -32386,7 +32386,7 @@
         <v>2018</v>
       </c>
       <c r="N528" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O528" t="s">
         <v>2031</v>
@@ -32918,7 +32918,7 @@
         <v>1893</v>
       </c>
       <c r="H539" t="s">
-        <v>1950</v>
+        <v>1949</v>
       </c>
       <c r="I539" t="s">
         <v>1995</v>
@@ -32936,7 +32936,7 @@
         <v>2018</v>
       </c>
       <c r="N539" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O539" t="s">
         <v>2031</v>
@@ -33130,7 +33130,7 @@
         <v>2018</v>
       </c>
       <c r="N543" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O543" t="s">
         <v>2029</v>
@@ -33180,7 +33180,7 @@
         <v>2016</v>
       </c>
       <c r="N544" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O544" t="s">
         <v>2029</v>
@@ -33256,7 +33256,7 @@
         <v>1893</v>
       </c>
       <c r="H546" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="I546" t="s">
         <v>1995</v>
@@ -33274,7 +33274,7 @@
         <v>2018</v>
       </c>
       <c r="N546" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O546" t="s">
         <v>2031</v>
@@ -33303,7 +33303,7 @@
         <v>1893</v>
       </c>
       <c r="H547" t="s">
-        <v>1955</v>
+        <v>1954</v>
       </c>
       <c r="I547" t="s">
         <v>1995</v>
@@ -33321,7 +33321,7 @@
         <v>2018</v>
       </c>
       <c r="N547" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O547" t="s">
         <v>2031</v>
@@ -33497,7 +33497,7 @@
         <v>1893</v>
       </c>
       <c r="H551" t="s">
-        <v>1943</v>
+        <v>1956</v>
       </c>
       <c r="I551" t="s">
         <v>1995</v>
@@ -33515,7 +33515,7 @@
         <v>2018</v>
       </c>
       <c r="N551" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O551" t="s">
         <v>2031</v>
@@ -33547,7 +33547,7 @@
         <v>1893</v>
       </c>
       <c r="H552" t="s">
-        <v>1943</v>
+        <v>1956</v>
       </c>
       <c r="I552" t="s">
         <v>1995</v>
@@ -33565,7 +33565,7 @@
         <v>2018</v>
       </c>
       <c r="N552" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O552" t="s">
         <v>2031</v>
@@ -33785,7 +33785,7 @@
         <v>1893</v>
       </c>
       <c r="H557" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="I557" t="s">
         <v>1995</v>
@@ -33803,7 +33803,7 @@
         <v>2018</v>
       </c>
       <c r="N557" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O557" t="s">
         <v>2031</v>
@@ -33829,7 +33829,7 @@
         <v>1893</v>
       </c>
       <c r="H558" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="I558" t="s">
         <v>1995</v>
@@ -33847,7 +33847,7 @@
         <v>2018</v>
       </c>
       <c r="N558" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O558" t="s">
         <v>2031</v>
@@ -33929,7 +33929,7 @@
         <v>1893</v>
       </c>
       <c r="H560" t="s">
-        <v>1943</v>
+        <v>1956</v>
       </c>
       <c r="I560" t="s">
         <v>1995</v>
@@ -33947,7 +33947,7 @@
         <v>2016</v>
       </c>
       <c r="N560" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O560" t="s">
         <v>2029</v>
@@ -34261,7 +34261,7 @@
         <v>1893</v>
       </c>
       <c r="H567" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="I567" t="s">
         <v>1995</v>
@@ -34279,7 +34279,7 @@
         <v>2018</v>
       </c>
       <c r="N567" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O567" t="s">
         <v>2031</v>
@@ -34311,7 +34311,7 @@
         <v>1893</v>
       </c>
       <c r="H568" t="s">
-        <v>1949</v>
+        <v>1948</v>
       </c>
       <c r="I568" t="s">
         <v>1989</v>
@@ -34423,7 +34423,7 @@
         <v>2018</v>
       </c>
       <c r="N570" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O570" t="s">
         <v>2031</v>
@@ -35287,7 +35287,7 @@
         <v>1893</v>
       </c>
       <c r="H588" t="s">
-        <v>1950</v>
+        <v>1949</v>
       </c>
       <c r="I588" t="s">
         <v>1995</v>
@@ -35305,7 +35305,7 @@
         <v>2018</v>
       </c>
       <c r="N588" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O588" t="s">
         <v>2031</v>
@@ -35337,7 +35337,7 @@
         <v>1893</v>
       </c>
       <c r="H589" t="s">
-        <v>1950</v>
+        <v>1949</v>
       </c>
       <c r="I589" t="s">
         <v>1995</v>
@@ -35355,7 +35355,7 @@
         <v>2018</v>
       </c>
       <c r="N589" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O589" t="s">
         <v>2031</v>
@@ -35455,7 +35455,7 @@
         <v>2018</v>
       </c>
       <c r="N591" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O591" t="s">
         <v>2031</v>
@@ -35505,7 +35505,7 @@
         <v>2018</v>
       </c>
       <c r="N592" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O592" t="s">
         <v>2029</v>
@@ -36187,7 +36187,7 @@
         <v>1893</v>
       </c>
       <c r="H606" t="s">
-        <v>1952</v>
+        <v>1951</v>
       </c>
       <c r="I606" t="s">
         <v>1995</v>
@@ -36205,7 +36205,7 @@
         <v>2017</v>
       </c>
       <c r="N606" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O606" t="s">
         <v>2031</v>
@@ -36237,7 +36237,7 @@
         <v>1893</v>
       </c>
       <c r="H607" t="s">
-        <v>1952</v>
+        <v>1951</v>
       </c>
       <c r="I607" t="s">
         <v>1995</v>
@@ -36255,7 +36255,7 @@
         <v>2018</v>
       </c>
       <c r="N607" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O607" t="s">
         <v>2029</v>
@@ -36731,7 +36731,7 @@
         <v>1893</v>
       </c>
       <c r="H617" t="s">
-        <v>1952</v>
+        <v>1951</v>
       </c>
       <c r="I617" t="s">
         <v>1995</v>
@@ -36749,7 +36749,7 @@
         <v>2016</v>
       </c>
       <c r="N617" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O617" t="s">
         <v>2031</v>
@@ -37248,7 +37248,7 @@
         <v>1893</v>
       </c>
       <c r="H628" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="I628" t="s">
         <v>1995</v>
@@ -37266,7 +37266,7 @@
         <v>2018</v>
       </c>
       <c r="N628" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O628" t="s">
         <v>2031</v>
@@ -37316,7 +37316,7 @@
         <v>2018</v>
       </c>
       <c r="N629" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O629" t="s">
         <v>2031</v>
@@ -37466,7 +37466,7 @@
         <v>2018</v>
       </c>
       <c r="N632" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O632" t="s">
         <v>2031</v>
@@ -37936,7 +37936,7 @@
         <v>2018</v>
       </c>
       <c r="N642" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O642" t="s">
         <v>2031</v>
@@ -37983,7 +37983,7 @@
         <v>2018</v>
       </c>
       <c r="N643" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O643" t="s">
         <v>2031</v>
@@ -38012,7 +38012,7 @@
         <v>1893</v>
       </c>
       <c r="H644" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="I644" t="s">
         <v>1995</v>
@@ -38030,7 +38030,7 @@
         <v>2018</v>
       </c>
       <c r="N644" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O644" t="s">
         <v>2029</v>
@@ -38077,7 +38077,7 @@
         <v>2018</v>
       </c>
       <c r="N645" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O645" t="s">
         <v>2031</v>
@@ -38159,7 +38159,7 @@
         <v>1893</v>
       </c>
       <c r="H647" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="I647" t="s">
         <v>1995</v>
@@ -38177,7 +38177,7 @@
         <v>2018</v>
       </c>
       <c r="N647" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O647" t="s">
         <v>2029</v>
@@ -38209,7 +38209,7 @@
         <v>1893</v>
       </c>
       <c r="H648" t="s">
-        <v>1952</v>
+        <v>1951</v>
       </c>
       <c r="I648" t="s">
         <v>1995</v>
@@ -38227,7 +38227,7 @@
         <v>2018</v>
       </c>
       <c r="N648" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O648" t="s">
         <v>2029</v>
@@ -38259,7 +38259,7 @@
         <v>1893</v>
       </c>
       <c r="H649" t="s">
-        <v>1952</v>
+        <v>1951</v>
       </c>
       <c r="I649" t="s">
         <v>1995</v>
@@ -38277,7 +38277,7 @@
         <v>2018</v>
       </c>
       <c r="N649" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O649" t="s">
         <v>2031</v>
@@ -38327,7 +38327,7 @@
         <v>2018</v>
       </c>
       <c r="N650" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O650" t="s">
         <v>2031</v>
@@ -38359,7 +38359,7 @@
         <v>1893</v>
       </c>
       <c r="H651" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="I651" t="s">
         <v>1995</v>
@@ -38377,7 +38377,7 @@
         <v>2019</v>
       </c>
       <c r="N651" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O651" t="s">
         <v>2029</v>
@@ -38403,7 +38403,7 @@
         <v>1893</v>
       </c>
       <c r="H652" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="I652" t="s">
         <v>1995</v>
@@ -38421,7 +38421,7 @@
         <v>2019</v>
       </c>
       <c r="N652" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O652" t="s">
         <v>2029</v>
@@ -38447,7 +38447,7 @@
         <v>1893</v>
       </c>
       <c r="H653" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="I653" t="s">
         <v>1995</v>
@@ -38465,7 +38465,7 @@
         <v>2019</v>
       </c>
       <c r="N653" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O653" t="s">
         <v>2029</v>
@@ -38697,7 +38697,7 @@
         <v>1893</v>
       </c>
       <c r="H658" t="s">
-        <v>1955</v>
+        <v>1954</v>
       </c>
       <c r="I658" t="s">
         <v>1995</v>
@@ -38715,7 +38715,7 @@
         <v>2018</v>
       </c>
       <c r="N658" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O658" t="s">
         <v>2031</v>
@@ -38747,7 +38747,7 @@
         <v>1893</v>
       </c>
       <c r="H659" t="s">
-        <v>1955</v>
+        <v>1954</v>
       </c>
       <c r="I659" t="s">
         <v>1995</v>
@@ -38765,7 +38765,7 @@
         <v>2018</v>
       </c>
       <c r="N659" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O659" t="s">
         <v>2031</v>
@@ -38997,7 +38997,7 @@
         <v>1893</v>
       </c>
       <c r="H664" t="s">
-        <v>1950</v>
+        <v>1949</v>
       </c>
       <c r="I664" t="s">
         <v>1995</v>
@@ -39015,7 +39015,7 @@
         <v>2018</v>
       </c>
       <c r="N664" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O664" t="s">
         <v>2031</v>
@@ -39244,7 +39244,7 @@
         <v>1893</v>
       </c>
       <c r="H669" t="s">
-        <v>1955</v>
+        <v>1954</v>
       </c>
       <c r="I669" t="s">
         <v>1995</v>
@@ -39262,7 +39262,7 @@
         <v>2018</v>
       </c>
       <c r="N669" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O669" t="s">
         <v>2031</v>
@@ -39603,7 +39603,7 @@
         <v>2018</v>
       </c>
       <c r="N676" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O676" t="s">
         <v>2031</v>
@@ -40699,7 +40699,7 @@
         <v>1893</v>
       </c>
       <c r="H699" t="s">
-        <v>1953</v>
+        <v>1952</v>
       </c>
       <c r="I699" t="s">
         <v>1995</v>
@@ -40717,7 +40717,7 @@
         <v>2018</v>
       </c>
       <c r="N699" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O699" t="s">
         <v>2031</v>
@@ -40914,7 +40914,7 @@
         <v>2016</v>
       </c>
       <c r="N703" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O703" t="s">
         <v>2031</v>
@@ -41043,7 +41043,7 @@
         <v>1893</v>
       </c>
       <c r="H706" t="s">
-        <v>1954</v>
+        <v>1953</v>
       </c>
       <c r="I706" t="s">
         <v>1995</v>
@@ -41061,7 +41061,7 @@
         <v>2018</v>
       </c>
       <c r="N706" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O706" t="s">
         <v>2031</v>
@@ -41093,7 +41093,7 @@
         <v>1893</v>
       </c>
       <c r="H707" t="s">
-        <v>1943</v>
+        <v>1956</v>
       </c>
       <c r="I707" t="s">
         <v>1995</v>
@@ -41111,7 +41111,7 @@
         <v>2018</v>
       </c>
       <c r="N707" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O707" t="s">
         <v>2031</v>
@@ -41193,7 +41193,7 @@
         <v>1893</v>
       </c>
       <c r="H709" t="s">
-        <v>1949</v>
+        <v>1948</v>
       </c>
       <c r="I709" t="s">
         <v>1989</v>
@@ -41240,7 +41240,7 @@
         <v>1893</v>
       </c>
       <c r="H710" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="I710" t="s">
         <v>1995</v>
@@ -41258,7 +41258,7 @@
         <v>2019</v>
       </c>
       <c r="N710" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O710" t="s">
         <v>2029</v>
@@ -41340,7 +41340,7 @@
         <v>1893</v>
       </c>
       <c r="H712" t="s">
-        <v>1946</v>
+        <v>1945</v>
       </c>
       <c r="I712" t="s">
         <v>1995</v>
@@ -41358,7 +41358,7 @@
         <v>2017</v>
       </c>
       <c r="N712" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O712" t="s">
         <v>2031</v>
@@ -41590,7 +41590,7 @@
         <v>1893</v>
       </c>
       <c r="H717" t="s">
-        <v>1949</v>
+        <v>1948</v>
       </c>
       <c r="I717" t="s">
         <v>1989</v>
@@ -41690,7 +41690,7 @@
         <v>1893</v>
       </c>
       <c r="H719" t="s">
-        <v>1946</v>
+        <v>1945</v>
       </c>
       <c r="I719" t="s">
         <v>1995</v>
@@ -41708,7 +41708,7 @@
         <v>2019</v>
       </c>
       <c r="N719" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O719" t="s">
         <v>2029</v>
@@ -41758,7 +41758,7 @@
         <v>2019</v>
       </c>
       <c r="N720" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O720" t="s">
         <v>2029</v>
@@ -41790,7 +41790,7 @@
         <v>1893</v>
       </c>
       <c r="H721" t="s">
-        <v>1952</v>
+        <v>1951</v>
       </c>
       <c r="I721" t="s">
         <v>1995</v>
@@ -41808,7 +41808,7 @@
         <v>2018</v>
       </c>
       <c r="N721" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O721" t="s">
         <v>2031</v>
@@ -41858,7 +41858,7 @@
         <v>2018</v>
       </c>
       <c r="N722" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O722" t="s">
         <v>2031</v>
@@ -42287,7 +42287,7 @@
         <v>1893</v>
       </c>
       <c r="H731" t="s">
-        <v>1950</v>
+        <v>1949</v>
       </c>
       <c r="I731" t="s">
         <v>1995</v>
@@ -42305,7 +42305,7 @@
         <v>2018</v>
       </c>
       <c r="N731" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O731" t="s">
         <v>2031</v>
@@ -42387,7 +42387,7 @@
         <v>1893</v>
       </c>
       <c r="H733" t="s">
-        <v>1951</v>
+        <v>1950</v>
       </c>
       <c r="I733" t="s">
         <v>1996</v>
@@ -42502,7 +42502,7 @@
         <v>2018</v>
       </c>
       <c r="N735" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O735" t="s">
         <v>2031</v>
@@ -42552,7 +42552,7 @@
         <v>2018</v>
       </c>
       <c r="N736" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O736" t="s">
         <v>2031</v>
@@ -42602,7 +42602,7 @@
         <v>2018</v>
       </c>
       <c r="N737" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O737" t="s">
         <v>2031</v>
@@ -42652,7 +42652,7 @@
         <v>2018</v>
       </c>
       <c r="N738" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O738" t="s">
         <v>2031</v>
@@ -42702,7 +42702,7 @@
         <v>2018</v>
       </c>
       <c r="N739" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O739" t="s">
         <v>2031</v>
@@ -42872,7 +42872,7 @@
         <v>1893</v>
       </c>
       <c r="H743" t="s">
-        <v>1950</v>
+        <v>1949</v>
       </c>
       <c r="I743" t="s">
         <v>1995</v>
@@ -42890,7 +42890,7 @@
         <v>2018</v>
       </c>
       <c r="N743" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O743" t="s">
         <v>2031</v>
@@ -42922,7 +42922,7 @@
         <v>1893</v>
       </c>
       <c r="H744" t="s">
-        <v>1952</v>
+        <v>1951</v>
       </c>
       <c r="I744" t="s">
         <v>1995</v>
@@ -42940,7 +42940,7 @@
         <v>2019</v>
       </c>
       <c r="N744" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O744" t="s">
         <v>2029</v>
@@ -42972,7 +42972,7 @@
         <v>1893</v>
       </c>
       <c r="H745" t="s">
-        <v>1952</v>
+        <v>1951</v>
       </c>
       <c r="I745" t="s">
         <v>1995</v>
@@ -42990,7 +42990,7 @@
         <v>2019</v>
       </c>
       <c r="N745" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O745" t="s">
         <v>2029</v>
@@ -43137,7 +43137,7 @@
         <v>2018</v>
       </c>
       <c r="N748" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O748" t="s">
         <v>2029</v>
@@ -43169,7 +43169,7 @@
         <v>1893</v>
       </c>
       <c r="H749" t="s">
-        <v>1947</v>
+        <v>1946</v>
       </c>
       <c r="I749" t="s">
         <v>1992</v>
@@ -43269,7 +43269,7 @@
         <v>1893</v>
       </c>
       <c r="H751" t="s">
-        <v>1947</v>
+        <v>1946</v>
       </c>
       <c r="I751" t="s">
         <v>1992</v>
@@ -43316,7 +43316,7 @@
         <v>1893</v>
       </c>
       <c r="H752" t="s">
-        <v>1949</v>
+        <v>1948</v>
       </c>
       <c r="I752" t="s">
         <v>1989</v>
@@ -43384,7 +43384,7 @@
         <v>2018</v>
       </c>
       <c r="N753" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O753" t="s">
         <v>2031</v>
@@ -43434,7 +43434,7 @@
         <v>2018</v>
       </c>
       <c r="N754" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O754" t="s">
         <v>2031</v>
@@ -43657,7 +43657,7 @@
         <v>1893</v>
       </c>
       <c r="H759" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="I759" t="s">
         <v>1995</v>
@@ -43675,7 +43675,7 @@
         <v>2018</v>
       </c>
       <c r="N759" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O759" t="s">
         <v>2031</v>
@@ -43707,7 +43707,7 @@
         <v>1893</v>
       </c>
       <c r="H760" t="s">
-        <v>1955</v>
+        <v>1954</v>
       </c>
       <c r="I760" t="s">
         <v>1995</v>
@@ -43725,7 +43725,7 @@
         <v>2018</v>
       </c>
       <c r="N760" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O760" t="s">
         <v>2029</v>
@@ -43854,7 +43854,7 @@
         <v>1893</v>
       </c>
       <c r="H763" t="s">
-        <v>1954</v>
+        <v>1953</v>
       </c>
       <c r="I763" t="s">
         <v>1995</v>
@@ -43872,7 +43872,7 @@
         <v>2018</v>
       </c>
       <c r="N763" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O763" t="s">
         <v>2031</v>
@@ -43954,7 +43954,7 @@
         <v>1893</v>
       </c>
       <c r="H765" t="s">
-        <v>1948</v>
+        <v>1947</v>
       </c>
       <c r="I765" t="s">
         <v>1997</v>
@@ -44051,7 +44051,7 @@
         <v>1893</v>
       </c>
       <c r="H767" t="s">
-        <v>1943</v>
+        <v>1956</v>
       </c>
       <c r="I767" t="s">
         <v>1995</v>
@@ -44069,7 +44069,7 @@
         <v>2018</v>
       </c>
       <c r="N767" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O767" t="s">
         <v>2029</v>
@@ -44169,7 +44169,7 @@
         <v>2018</v>
       </c>
       <c r="N769" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O769" t="s">
         <v>2031</v>
@@ -44266,7 +44266,7 @@
         <v>2018</v>
       </c>
       <c r="N771" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O771" t="s">
         <v>2031</v>
@@ -44298,7 +44298,7 @@
         <v>1893</v>
       </c>
       <c r="H772" t="s">
-        <v>1953</v>
+        <v>1952</v>
       </c>
       <c r="I772" t="s">
         <v>1995</v>
@@ -44316,7 +44316,7 @@
         <v>2018</v>
       </c>
       <c r="N772" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O772" t="s">
         <v>2031</v>
@@ -44795,7 +44795,7 @@
         <v>1893</v>
       </c>
       <c r="H782" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="I782" t="s">
         <v>1995</v>
@@ -44813,7 +44813,7 @@
         <v>2016</v>
       </c>
       <c r="N782" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O782" t="s">
         <v>2031</v>
@@ -44842,7 +44842,7 @@
         <v>1893</v>
       </c>
       <c r="H783" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="I783" t="s">
         <v>1995</v>
@@ -44860,7 +44860,7 @@
         <v>2018</v>
       </c>
       <c r="N783" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O783" t="s">
         <v>2029</v>
@@ -44951,7 +44951,7 @@
         <v>2018</v>
       </c>
       <c r="N785" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O785" t="s">
         <v>2031</v>
@@ -45001,7 +45001,7 @@
         <v>2016</v>
       </c>
       <c r="N786" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O786" t="s">
         <v>2029</v>
@@ -45051,7 +45051,7 @@
         <v>2016</v>
       </c>
       <c r="N787" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O787" t="s">
         <v>2031</v>
@@ -45101,7 +45101,7 @@
         <v>2018</v>
       </c>
       <c r="N788" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O788" t="s">
         <v>2031</v>
@@ -45174,7 +45174,7 @@
         <v>1893</v>
       </c>
       <c r="H790" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="I790" t="s">
         <v>1995</v>
@@ -45192,7 +45192,7 @@
         <v>2019</v>
       </c>
       <c r="N790" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O790" t="s">
         <v>2029</v>
@@ -45392,7 +45392,7 @@
         <v>2016</v>
       </c>
       <c r="N794" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O794" t="s">
         <v>2031</v>
@@ -45794,7 +45794,7 @@
         <v>1893</v>
       </c>
       <c r="H803" t="s">
-        <v>1949</v>
+        <v>1948</v>
       </c>
       <c r="I803" t="s">
         <v>1989</v>
@@ -45844,7 +45844,7 @@
         <v>1893</v>
       </c>
       <c r="H804" t="s">
-        <v>1949</v>
+        <v>1948</v>
       </c>
       <c r="I804" t="s">
         <v>1989</v>
@@ -45894,7 +45894,7 @@
         <v>1893</v>
       </c>
       <c r="H805" t="s">
-        <v>1949</v>
+        <v>1948</v>
       </c>
       <c r="I805" t="s">
         <v>1989</v>
@@ -45944,7 +45944,7 @@
         <v>1893</v>
       </c>
       <c r="H806" t="s">
-        <v>1943</v>
+        <v>1956</v>
       </c>
       <c r="I806" t="s">
         <v>1995</v>
@@ -45962,7 +45962,7 @@
         <v>2018</v>
       </c>
       <c r="N806" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O806" t="s">
         <v>2031</v>
@@ -46209,7 +46209,7 @@
         <v>2018</v>
       </c>
       <c r="N811" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O811" t="s">
         <v>2031</v>
@@ -46473,7 +46473,7 @@
         <v>1893</v>
       </c>
       <c r="H817" t="s">
-        <v>1953</v>
+        <v>1952</v>
       </c>
       <c r="I817" t="s">
         <v>1995</v>
@@ -46491,7 +46491,7 @@
         <v>2018</v>
       </c>
       <c r="N817" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O817" t="s">
         <v>2031</v>
@@ -46591,7 +46591,7 @@
         <v>2018</v>
       </c>
       <c r="N819" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O819" t="s">
         <v>2031</v>
@@ -46691,7 +46691,7 @@
         <v>2018</v>
       </c>
       <c r="N821" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O821" t="s">
         <v>2029</v>
@@ -46717,7 +46717,7 @@
         <v>1893</v>
       </c>
       <c r="H822" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="I822" t="s">
         <v>1995</v>
@@ -46735,7 +46735,7 @@
         <v>2019</v>
       </c>
       <c r="N822" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O822" t="s">
         <v>2029</v>
@@ -46782,7 +46782,7 @@
         <v>2018</v>
       </c>
       <c r="N823" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O823" t="s">
         <v>2029</v>
@@ -46929,7 +46929,7 @@
         <v>2018</v>
       </c>
       <c r="N826" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O826" t="s">
         <v>2031</v>
@@ -46961,7 +46961,7 @@
         <v>1893</v>
       </c>
       <c r="H827" t="s">
-        <v>1947</v>
+        <v>1946</v>
       </c>
       <c r="I827" t="s">
         <v>1992</v>
@@ -47211,7 +47211,7 @@
         <v>2018</v>
       </c>
       <c r="N832" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O832" t="s">
         <v>2031</v>
@@ -47261,7 +47261,7 @@
         <v>2018</v>
       </c>
       <c r="N833" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O833" t="s">
         <v>2031</v>
@@ -47311,7 +47311,7 @@
         <v>2018</v>
       </c>
       <c r="N834" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O834" t="s">
         <v>2031</v>
@@ -47361,7 +47361,7 @@
         <v>2018</v>
       </c>
       <c r="N835" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O835" t="s">
         <v>2031</v>
@@ -47411,7 +47411,7 @@
         <v>2018</v>
       </c>
       <c r="N836" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O836" t="s">
         <v>2031</v>
@@ -47461,7 +47461,7 @@
         <v>2016</v>
       </c>
       <c r="N837" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O837" t="s">
         <v>2029</v>
@@ -47511,7 +47511,7 @@
         <v>2018</v>
       </c>
       <c r="N838" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O838" t="s">
         <v>2029</v>
@@ -47693,7 +47693,7 @@
         <v>1893</v>
       </c>
       <c r="H842" t="s">
-        <v>1953</v>
+        <v>1952</v>
       </c>
       <c r="I842" t="s">
         <v>1995</v>
@@ -47711,7 +47711,7 @@
         <v>2016</v>
       </c>
       <c r="N842" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O842" t="s">
         <v>2029</v>
@@ -47811,7 +47811,7 @@
         <v>2018</v>
       </c>
       <c r="N844" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O844" t="s">
         <v>2031</v>
@@ -47843,7 +47843,7 @@
         <v>1893</v>
       </c>
       <c r="H845" t="s">
-        <v>1951</v>
+        <v>1950</v>
       </c>
       <c r="I845" t="s">
         <v>1996</v>
@@ -48331,7 +48331,7 @@
         <v>1893</v>
       </c>
       <c r="H855" t="s">
-        <v>1955</v>
+        <v>1954</v>
       </c>
       <c r="I855" t="s">
         <v>1995</v>
@@ -48349,7 +48349,7 @@
         <v>2018</v>
       </c>
       <c r="N855" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O855" t="s">
         <v>2029</v>
@@ -48481,7 +48481,7 @@
         <v>1893</v>
       </c>
       <c r="H858" t="s">
-        <v>1947</v>
+        <v>1946</v>
       </c>
       <c r="I858" t="s">
         <v>1992</v>
@@ -48531,7 +48531,7 @@
         <v>1893</v>
       </c>
       <c r="H859" t="s">
-        <v>1947</v>
+        <v>1946</v>
       </c>
       <c r="I859" t="s">
         <v>1992</v>
@@ -48816,7 +48816,7 @@
         <v>1893</v>
       </c>
       <c r="H865" t="s">
-        <v>1954</v>
+        <v>1953</v>
       </c>
       <c r="I865" t="s">
         <v>1995</v>
@@ -48834,7 +48834,7 @@
         <v>2019</v>
       </c>
       <c r="N865" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O865" t="s">
         <v>2029</v>
@@ -48863,7 +48863,7 @@
         <v>1893</v>
       </c>
       <c r="H866" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="I866" t="s">
         <v>1995</v>
@@ -48881,7 +48881,7 @@
         <v>2017</v>
       </c>
       <c r="N866" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O866" t="s">
         <v>2031</v>
@@ -48910,7 +48910,7 @@
         <v>1893</v>
       </c>
       <c r="H867" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="I867" t="s">
         <v>1995</v>
@@ -48928,7 +48928,7 @@
         <v>2018</v>
       </c>
       <c r="N867" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O867" t="s">
         <v>2031</v>
@@ -48978,7 +48978,7 @@
         <v>2016</v>
       </c>
       <c r="N868" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O868" t="s">
         <v>2029</v>
@@ -49010,7 +49010,7 @@
         <v>1893</v>
       </c>
       <c r="H869" t="s">
-        <v>1943</v>
+        <v>1956</v>
       </c>
       <c r="I869" t="s">
         <v>1995</v>
@@ -49028,7 +49028,7 @@
         <v>2018</v>
       </c>
       <c r="N869" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O869" t="s">
         <v>2031</v>
@@ -49416,7 +49416,7 @@
         <v>2018</v>
       </c>
       <c r="N877" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O877" t="s">
         <v>2031</v>
@@ -49498,7 +49498,7 @@
         <v>1893</v>
       </c>
       <c r="H879" t="s">
-        <v>1954</v>
+        <v>1953</v>
       </c>
       <c r="I879" t="s">
         <v>1995</v>
@@ -49516,7 +49516,7 @@
         <v>2019</v>
       </c>
       <c r="N879" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O879" t="s">
         <v>2029</v>
@@ -49545,7 +49545,7 @@
         <v>1893</v>
       </c>
       <c r="H880" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="I880" t="s">
         <v>1995</v>
@@ -49563,7 +49563,7 @@
         <v>2018</v>
       </c>
       <c r="N880" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O880" t="s">
         <v>2031</v>
@@ -49642,7 +49642,7 @@
         <v>1893</v>
       </c>
       <c r="H882" t="s">
-        <v>1955</v>
+        <v>1954</v>
       </c>
       <c r="I882" t="s">
         <v>1995</v>
@@ -49660,7 +49660,7 @@
         <v>2018</v>
       </c>
       <c r="N882" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O882" t="s">
         <v>2031</v>
@@ -49692,7 +49692,7 @@
         <v>1893</v>
       </c>
       <c r="H883" t="s">
-        <v>1950</v>
+        <v>1949</v>
       </c>
       <c r="I883" t="s">
         <v>1995</v>
@@ -49710,7 +49710,7 @@
         <v>2018</v>
       </c>
       <c r="N883" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O883" t="s">
         <v>2031</v>
@@ -49742,7 +49742,7 @@
         <v>1893</v>
       </c>
       <c r="H884" t="s">
-        <v>1950</v>
+        <v>1949</v>
       </c>
       <c r="I884" t="s">
         <v>1995</v>
@@ -49760,7 +49760,7 @@
         <v>2018</v>
       </c>
       <c r="N884" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O884" t="s">
         <v>2031</v>
@@ -49883,7 +49883,7 @@
         <v>1893</v>
       </c>
       <c r="H887" t="s">
-        <v>1955</v>
+        <v>1954</v>
       </c>
       <c r="I887" t="s">
         <v>1995</v>
@@ -49901,7 +49901,7 @@
         <v>2018</v>
       </c>
       <c r="N887" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O887" t="s">
         <v>2031</v>
@@ -49983,7 +49983,7 @@
         <v>1893</v>
       </c>
       <c r="H889" t="s">
-        <v>1949</v>
+        <v>1948</v>
       </c>
       <c r="I889" t="s">
         <v>1989</v>
@@ -50033,7 +50033,7 @@
         <v>1893</v>
       </c>
       <c r="H890" t="s">
-        <v>1943</v>
+        <v>1956</v>
       </c>
       <c r="I890" t="s">
         <v>1995</v>
@@ -50051,7 +50051,7 @@
         <v>2018</v>
       </c>
       <c r="N890" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O890" t="s">
         <v>2029</v>
@@ -50145,7 +50145,7 @@
         <v>2018</v>
       </c>
       <c r="N892" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O892" t="s">
         <v>2029</v>
@@ -50442,7 +50442,7 @@
         <v>2017</v>
       </c>
       <c r="N898" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O898" t="s">
         <v>2031</v>
@@ -50474,7 +50474,7 @@
         <v>1893</v>
       </c>
       <c r="H899" t="s">
-        <v>1949</v>
+        <v>1948</v>
       </c>
       <c r="I899" t="s">
         <v>1989</v>
@@ -50521,7 +50521,7 @@
         <v>1893</v>
       </c>
       <c r="H900" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="I900" t="s">
         <v>1995</v>
@@ -50539,7 +50539,7 @@
         <v>2017</v>
       </c>
       <c r="N900" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O900" t="s">
         <v>2031</v>
@@ -50565,7 +50565,7 @@
         <v>1893</v>
       </c>
       <c r="H901" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="I901" t="s">
         <v>1995</v>
@@ -50583,7 +50583,7 @@
         <v>2018</v>
       </c>
       <c r="N901" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O901" t="s">
         <v>2031</v>
@@ -50633,7 +50633,7 @@
         <v>2016</v>
       </c>
       <c r="N902" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O902" t="s">
         <v>2031</v>
@@ -50680,7 +50680,7 @@
         <v>2018</v>
       </c>
       <c r="N903" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O903" t="s">
         <v>2029</v>
@@ -50727,7 +50727,7 @@
         <v>2018</v>
       </c>
       <c r="N904" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O904" t="s">
         <v>2029</v>
@@ -50806,7 +50806,7 @@
         <v>1893</v>
       </c>
       <c r="H906" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="I906" t="s">
         <v>1995</v>
@@ -50824,7 +50824,7 @@
         <v>2016</v>
       </c>
       <c r="N906" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O906" t="s">
         <v>2029</v>
@@ -51174,7 +51174,7 @@
         <v>2017</v>
       </c>
       <c r="N913" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O913" t="s">
         <v>2031</v>
@@ -51224,7 +51224,7 @@
         <v>2018</v>
       </c>
       <c r="N914" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O914" t="s">
         <v>2031</v>
@@ -51274,7 +51274,7 @@
         <v>2017</v>
       </c>
       <c r="N915" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O915" t="s">
         <v>2031</v>
@@ -51324,7 +51324,7 @@
         <v>2017</v>
       </c>
       <c r="N916" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O916" t="s">
         <v>2031</v>
@@ -51453,7 +51453,7 @@
         <v>1893</v>
       </c>
       <c r="H919" t="s">
-        <v>1954</v>
+        <v>1953</v>
       </c>
       <c r="I919" t="s">
         <v>1995</v>
@@ -51471,7 +51471,7 @@
         <v>2018</v>
       </c>
       <c r="N919" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O919" t="s">
         <v>2031</v>
@@ -51841,7 +51841,7 @@
         <v>1893</v>
       </c>
       <c r="H927" t="s">
-        <v>1949</v>
+        <v>1948</v>
       </c>
       <c r="I927" t="s">
         <v>1989</v>
@@ -51891,7 +51891,7 @@
         <v>1893</v>
       </c>
       <c r="H928" t="s">
-        <v>1949</v>
+        <v>1948</v>
       </c>
       <c r="I928" t="s">
         <v>1989</v>
@@ -52632,7 +52632,7 @@
         <v>2018</v>
       </c>
       <c r="N943" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O943" t="s">
         <v>2031</v>
@@ -52711,7 +52711,7 @@
         <v>1893</v>
       </c>
       <c r="H945" t="s">
-        <v>1956</v>
+        <v>1955</v>
       </c>
       <c r="I945" t="s">
         <v>1995</v>
@@ -52729,7 +52729,7 @@
         <v>2016</v>
       </c>
       <c r="N945" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O945" t="s">
         <v>2031</v>
@@ -52914,7 +52914,7 @@
         <v>2016</v>
       </c>
       <c r="N949" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O949" t="s">
         <v>2031</v>
@@ -52961,7 +52961,7 @@
         <v>2016</v>
       </c>
       <c r="N950" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O950" t="s">
         <v>2031</v>
@@ -53008,7 +53008,7 @@
         <v>2016</v>
       </c>
       <c r="N951" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O951" t="s">
         <v>2031</v>
@@ -53278,7 +53278,7 @@
         <v>1893</v>
       </c>
       <c r="H957" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="I957" t="s">
         <v>1995</v>
@@ -53296,7 +53296,7 @@
         <v>2018</v>
       </c>
       <c r="N957" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O957" t="s">
         <v>2031</v>
@@ -53975,7 +53975,7 @@
         <v>2018</v>
       </c>
       <c r="N971" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O971" t="s">
         <v>2029</v>
@@ -54148,7 +54148,7 @@
         <v>1893</v>
       </c>
       <c r="H975" t="s">
-        <v>1952</v>
+        <v>1951</v>
       </c>
       <c r="I975" t="s">
         <v>1995</v>
@@ -54166,7 +54166,7 @@
         <v>2016</v>
       </c>
       <c r="N975" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O975" t="s">
         <v>2031</v>
@@ -54398,7 +54398,7 @@
         <v>1893</v>
       </c>
       <c r="H980" t="s">
-        <v>1956</v>
+        <v>1955</v>
       </c>
       <c r="I980" t="s">
         <v>1995</v>
@@ -54416,7 +54416,7 @@
         <v>2016</v>
       </c>
       <c r="N980" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O980" t="s">
         <v>2031</v>
@@ -54448,7 +54448,7 @@
         <v>1893</v>
       </c>
       <c r="H981" t="s">
-        <v>1955</v>
+        <v>1954</v>
       </c>
       <c r="I981" t="s">
         <v>1995</v>
@@ -54466,7 +54466,7 @@
         <v>2018</v>
       </c>
       <c r="N981" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O981" t="s">
         <v>2031</v>
@@ -54516,7 +54516,7 @@
         <v>2018</v>
       </c>
       <c r="N982" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O982" t="s">
         <v>2029</v>
@@ -54598,7 +54598,7 @@
         <v>1893</v>
       </c>
       <c r="H984" t="s">
-        <v>1949</v>
+        <v>1948</v>
       </c>
       <c r="I984" t="s">
         <v>1989</v>
@@ -54642,7 +54642,7 @@
         <v>1893</v>
       </c>
       <c r="H985" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="I985" t="s">
         <v>1995</v>
@@ -54660,7 +54660,7 @@
         <v>2016</v>
       </c>
       <c r="N985" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O985" t="s">
         <v>2029</v>
@@ -54710,7 +54710,7 @@
         <v>2018</v>
       </c>
       <c r="N986" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O986" t="s">
         <v>2029</v>
@@ -54760,7 +54760,7 @@
         <v>2018</v>
       </c>
       <c r="N987" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O987" t="s">
         <v>2031</v>
@@ -54810,7 +54810,7 @@
         <v>2018</v>
       </c>
       <c r="N988" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O988" t="s">
         <v>2031</v>
@@ -54860,7 +54860,7 @@
         <v>2018</v>
       </c>
       <c r="N989" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O989" t="s">
         <v>2031</v>
@@ -54889,7 +54889,7 @@
         <v>1893</v>
       </c>
       <c r="H990" t="s">
-        <v>1943</v>
+        <v>1956</v>
       </c>
       <c r="I990" t="s">
         <v>1995</v>
@@ -54907,7 +54907,7 @@
         <v>2018</v>
       </c>
       <c r="N990" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O990" t="s">
         <v>2031</v>
@@ -54957,7 +54957,7 @@
         <v>2016</v>
       </c>
       <c r="N991" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O991" t="s">
         <v>2031</v>
@@ -55039,7 +55039,7 @@
         <v>1893</v>
       </c>
       <c r="H993" t="s">
-        <v>1954</v>
+        <v>1953</v>
       </c>
       <c r="I993" t="s">
         <v>1995</v>
@@ -55057,7 +55057,7 @@
         <v>2016</v>
       </c>
       <c r="N993" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O993" t="s">
         <v>2031</v>
@@ -55539,7 +55539,7 @@
         <v>2018</v>
       </c>
       <c r="N1003" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O1003" t="s">
         <v>2031</v>
@@ -55589,7 +55589,7 @@
         <v>2018</v>
       </c>
       <c r="N1004" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O1004" t="s">
         <v>2031</v>
@@ -55665,7 +55665,7 @@
         <v>1893</v>
       </c>
       <c r="H1006" t="s">
-        <v>1955</v>
+        <v>1954</v>
       </c>
       <c r="I1006" t="s">
         <v>1995</v>
@@ -55683,7 +55683,7 @@
         <v>2016</v>
       </c>
       <c r="N1006" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O1006" t="s">
         <v>2029</v>
@@ -55815,7 +55815,7 @@
         <v>1893</v>
       </c>
       <c r="H1009" t="s">
-        <v>1955</v>
+        <v>1954</v>
       </c>
       <c r="I1009" t="s">
         <v>1995</v>
@@ -55833,7 +55833,7 @@
         <v>2018</v>
       </c>
       <c r="N1009" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O1009" t="s">
         <v>2031</v>
@@ -55865,7 +55865,7 @@
         <v>1893</v>
       </c>
       <c r="H1010" t="s">
-        <v>1947</v>
+        <v>1946</v>
       </c>
       <c r="I1010" t="s">
         <v>1992</v>
@@ -56065,7 +56065,7 @@
         <v>1893</v>
       </c>
       <c r="H1014" t="s">
-        <v>1949</v>
+        <v>1948</v>
       </c>
       <c r="I1014" t="s">
         <v>1989</v>
@@ -56215,7 +56215,7 @@
         <v>1893</v>
       </c>
       <c r="H1017" t="s">
-        <v>1949</v>
+        <v>1948</v>
       </c>
       <c r="I1017" t="s">
         <v>1989</v>
@@ -56365,7 +56365,7 @@
         <v>1893</v>
       </c>
       <c r="H1020" t="s">
-        <v>1952</v>
+        <v>1951</v>
       </c>
       <c r="I1020" t="s">
         <v>1995</v>
@@ -56383,7 +56383,7 @@
         <v>2018</v>
       </c>
       <c r="N1020" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O1020" t="s">
         <v>2031</v>
@@ -56415,7 +56415,7 @@
         <v>1893</v>
       </c>
       <c r="H1021" t="s">
-        <v>1952</v>
+        <v>1951</v>
       </c>
       <c r="I1021" t="s">
         <v>1995</v>
@@ -56433,7 +56433,7 @@
         <v>2018</v>
       </c>
       <c r="N1021" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O1021" t="s">
         <v>2031</v>
@@ -56624,7 +56624,7 @@
         <v>2016</v>
       </c>
       <c r="N1025" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O1025" t="s">
         <v>2031</v>
@@ -56656,7 +56656,7 @@
         <v>1893</v>
       </c>
       <c r="H1026" t="s">
-        <v>1950</v>
+        <v>1949</v>
       </c>
       <c r="I1026" t="s">
         <v>1995</v>
@@ -56674,7 +56674,7 @@
         <v>2018</v>
       </c>
       <c r="N1026" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O1026" t="s">
         <v>2031</v>
@@ -56700,7 +56700,7 @@
         <v>1893</v>
       </c>
       <c r="H1027" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="I1027" t="s">
         <v>1995</v>
@@ -56718,7 +56718,7 @@
         <v>2018</v>
       </c>
       <c r="N1027" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O1027" t="s">
         <v>2031</v>
@@ -56900,7 +56900,7 @@
         <v>1893</v>
       </c>
       <c r="H1031" t="s">
-        <v>1949</v>
+        <v>1948</v>
       </c>
       <c r="I1031" t="s">
         <v>1989</v>
@@ -56968,7 +56968,7 @@
         <v>2018</v>
       </c>
       <c r="N1032" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O1032" t="s">
         <v>2031</v>
@@ -57206,7 +57206,7 @@
         <v>2019</v>
       </c>
       <c r="N1037" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O1037" t="s">
         <v>2029</v>
@@ -57282,7 +57282,7 @@
         <v>1893</v>
       </c>
       <c r="H1039" t="s">
-        <v>1943</v>
+        <v>1956</v>
       </c>
       <c r="I1039" t="s">
         <v>1995</v>
@@ -57300,7 +57300,7 @@
         <v>2018</v>
       </c>
       <c r="N1039" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O1039" t="s">
         <v>2031</v>
@@ -57476,7 +57476,7 @@
         <v>1893</v>
       </c>
       <c r="H1043" t="s">
-        <v>1949</v>
+        <v>1948</v>
       </c>
       <c r="I1043" t="s">
         <v>1989</v>
@@ -57626,7 +57626,7 @@
         <v>1893</v>
       </c>
       <c r="H1046" t="s">
-        <v>1949</v>
+        <v>1948</v>
       </c>
       <c r="I1046" t="s">
         <v>1989</v>
@@ -57694,7 +57694,7 @@
         <v>2016</v>
       </c>
       <c r="N1047" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O1047" t="s">
         <v>2031</v>
@@ -57873,7 +57873,7 @@
         <v>1893</v>
       </c>
       <c r="H1051" t="s">
-        <v>1956</v>
+        <v>1955</v>
       </c>
       <c r="I1051" t="s">
         <v>1995</v>
@@ -57891,7 +57891,7 @@
         <v>2016</v>
       </c>
       <c r="N1051" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O1051" t="s">
         <v>2029</v>
@@ -58146,7 +58146,7 @@
         <v>1893</v>
       </c>
       <c r="H1057" t="s">
-        <v>1955</v>
+        <v>1954</v>
       </c>
       <c r="I1057" t="s">
         <v>1995</v>
@@ -58164,7 +58164,7 @@
         <v>2018</v>
       </c>
       <c r="N1057" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O1057" t="s">
         <v>2031</v>
@@ -58680,7 +58680,7 @@
         <v>1893</v>
       </c>
       <c r="H1069" t="s">
-        <v>1953</v>
+        <v>1952</v>
       </c>
       <c r="I1069" t="s">
         <v>1995</v>
@@ -58698,7 +58698,7 @@
         <v>2019</v>
       </c>
       <c r="N1069" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O1069" t="s">
         <v>2029</v>
@@ -58748,7 +58748,7 @@
         <v>2018</v>
       </c>
       <c r="N1070" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O1070" t="s">
         <v>2031</v>
@@ -58780,7 +58780,7 @@
         <v>1893</v>
       </c>
       <c r="H1071" t="s">
-        <v>1955</v>
+        <v>1954</v>
       </c>
       <c r="I1071" t="s">
         <v>1995</v>
@@ -58798,7 +58798,7 @@
         <v>2016</v>
       </c>
       <c r="N1071" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O1071" t="s">
         <v>2031</v>
@@ -58830,7 +58830,7 @@
         <v>1893</v>
       </c>
       <c r="H1072" t="s">
-        <v>1955</v>
+        <v>1954</v>
       </c>
       <c r="I1072" t="s">
         <v>1995</v>
@@ -58848,7 +58848,7 @@
         <v>2016</v>
       </c>
       <c r="N1072" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O1072" t="s">
         <v>2031</v>
@@ -59024,7 +59024,7 @@
         <v>1893</v>
       </c>
       <c r="H1076" t="s">
-        <v>1949</v>
+        <v>1948</v>
       </c>
       <c r="I1076" t="s">
         <v>1989</v>
@@ -59171,7 +59171,7 @@
         <v>1893</v>
       </c>
       <c r="H1079" t="s">
-        <v>1943</v>
+        <v>1956</v>
       </c>
       <c r="I1079" t="s">
         <v>1995</v>
@@ -59189,7 +59189,7 @@
         <v>2018</v>
       </c>
       <c r="N1079" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O1079" t="s">
         <v>2031</v>
@@ -59221,7 +59221,7 @@
         <v>1893</v>
       </c>
       <c r="H1080" t="s">
-        <v>1943</v>
+        <v>1956</v>
       </c>
       <c r="I1080" t="s">
         <v>1995</v>
@@ -59239,7 +59239,7 @@
         <v>2016</v>
       </c>
       <c r="N1080" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O1080" t="s">
         <v>2029</v>
@@ -59268,7 +59268,7 @@
         <v>1893</v>
       </c>
       <c r="H1081" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="I1081" t="s">
         <v>1995</v>
@@ -59286,7 +59286,7 @@
         <v>2018</v>
       </c>
       <c r="N1081" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O1081" t="s">
         <v>2031</v>
@@ -59412,7 +59412,7 @@
         <v>1893</v>
       </c>
       <c r="H1084" t="s">
-        <v>1956</v>
+        <v>1955</v>
       </c>
       <c r="I1084" t="s">
         <v>1995</v>
@@ -59430,7 +59430,7 @@
         <v>2018</v>
       </c>
       <c r="N1084" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O1084" t="s">
         <v>2031</v>
@@ -59562,7 +59562,7 @@
         <v>1893</v>
       </c>
       <c r="H1087" t="s">
-        <v>1949</v>
+        <v>1948</v>
       </c>
       <c r="I1087" t="s">
         <v>1989</v>
@@ -59659,7 +59659,7 @@
         <v>1893</v>
       </c>
       <c r="H1089" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="I1089" t="s">
         <v>1995</v>
@@ -59677,7 +59677,7 @@
         <v>2018</v>
       </c>
       <c r="N1089" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O1089" t="s">
         <v>2031</v>
@@ -59809,7 +59809,7 @@
         <v>1893</v>
       </c>
       <c r="H1092" t="s">
-        <v>1956</v>
+        <v>1955</v>
       </c>
       <c r="I1092" t="s">
         <v>1995</v>
@@ -59827,7 +59827,7 @@
         <v>2016</v>
       </c>
       <c r="N1092" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O1092" t="s">
         <v>2031</v>
@@ -60306,7 +60306,7 @@
         <v>2018</v>
       </c>
       <c r="N1102" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O1102" t="s">
         <v>2029</v>
@@ -60338,7 +60338,7 @@
         <v>1893</v>
       </c>
       <c r="H1103" t="s">
-        <v>1947</v>
+        <v>1946</v>
       </c>
       <c r="I1103" t="s">
         <v>1992</v>
@@ -60435,7 +60435,7 @@
         <v>1893</v>
       </c>
       <c r="H1105" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="I1105" t="s">
         <v>1995</v>
@@ -60453,7 +60453,7 @@
         <v>2017</v>
       </c>
       <c r="N1105" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O1105" t="s">
         <v>2031</v>
@@ -60647,7 +60647,7 @@
         <v>2018</v>
       </c>
       <c r="N1109" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O1109" t="s">
         <v>2029</v>
@@ -60829,7 +60829,7 @@
         <v>1893</v>
       </c>
       <c r="H1113" t="s">
-        <v>1947</v>
+        <v>1946</v>
       </c>
       <c r="I1113" t="s">
         <v>1992</v>
@@ -60879,7 +60879,7 @@
         <v>1893</v>
       </c>
       <c r="H1114" t="s">
-        <v>1947</v>
+        <v>1946</v>
       </c>
       <c r="I1114" t="s">
         <v>1992</v>
@@ -61070,7 +61070,7 @@
         <v>1893</v>
       </c>
       <c r="H1118" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="I1118" t="s">
         <v>1995</v>
@@ -61088,7 +61088,7 @@
         <v>2018</v>
       </c>
       <c r="N1118" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O1118" t="s">
         <v>2029</v>
@@ -61285,7 +61285,7 @@
         <v>2018</v>
       </c>
       <c r="N1122" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O1122" t="s">
         <v>2029</v>
@@ -62366,7 +62366,7 @@
         <v>1893</v>
       </c>
       <c r="H1145" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="I1145" t="s">
         <v>1995</v>
@@ -62384,7 +62384,7 @@
         <v>2018</v>
       </c>
       <c r="N1145" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O1145" t="s">
         <v>2031</v>
@@ -62639,7 +62639,7 @@
         <v>1893</v>
       </c>
       <c r="H1151" t="s">
-        <v>1955</v>
+        <v>1954</v>
       </c>
       <c r="I1151" t="s">
         <v>1995</v>
@@ -62657,7 +62657,7 @@
         <v>2018</v>
       </c>
       <c r="N1151" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O1151" t="s">
         <v>2029</v>
@@ -63086,7 +63086,7 @@
         <v>1893</v>
       </c>
       <c r="H1160" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="I1160" t="s">
         <v>1995</v>
@@ -63104,7 +63104,7 @@
         <v>2018</v>
       </c>
       <c r="N1160" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O1160" t="s">
         <v>2029</v>
@@ -63136,7 +63136,7 @@
         <v>1893</v>
       </c>
       <c r="H1161" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="I1161" t="s">
         <v>1995</v>
@@ -63154,7 +63154,7 @@
         <v>2018</v>
       </c>
       <c r="N1161" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O1161" t="s">
         <v>2031</v>
@@ -63245,7 +63245,7 @@
         <v>2019</v>
       </c>
       <c r="N1163" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O1163" t="s">
         <v>2029</v>
@@ -63277,7 +63277,7 @@
         <v>1893</v>
       </c>
       <c r="H1164" t="s">
-        <v>1943</v>
+        <v>1956</v>
       </c>
       <c r="I1164" t="s">
         <v>1995</v>
@@ -63295,7 +63295,7 @@
         <v>2018</v>
       </c>
       <c r="N1164" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O1164" t="s">
         <v>2031</v>
@@ -63582,7 +63582,7 @@
         <v>1893</v>
       </c>
       <c r="H1171" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="I1171" t="s">
         <v>1995</v>
@@ -63600,7 +63600,7 @@
         <v>2018</v>
       </c>
       <c r="N1171" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O1171" t="s">
         <v>2031</v>
@@ -63626,7 +63626,7 @@
         <v>1893</v>
       </c>
       <c r="H1172" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="I1172" t="s">
         <v>1995</v>
@@ -63644,7 +63644,7 @@
         <v>2018</v>
       </c>
       <c r="N1172" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O1172" t="s">
         <v>2031</v>
@@ -63670,7 +63670,7 @@
         <v>1893</v>
       </c>
       <c r="H1173" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="I1173" t="s">
         <v>1995</v>
@@ -63688,7 +63688,7 @@
         <v>2018</v>
       </c>
       <c r="N1173" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O1173" t="s">
         <v>2031</v>
@@ -63714,7 +63714,7 @@
         <v>1893</v>
       </c>
       <c r="H1174" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="I1174" t="s">
         <v>1995</v>
@@ -63732,7 +63732,7 @@
         <v>2018</v>
       </c>
       <c r="N1174" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O1174" t="s">
         <v>2031</v>
@@ -63758,7 +63758,7 @@
         <v>1893</v>
       </c>
       <c r="H1175" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="I1175" t="s">
         <v>1995</v>
@@ -63776,7 +63776,7 @@
         <v>2018</v>
       </c>
       <c r="N1175" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O1175" t="s">
         <v>2031</v>
@@ -63802,7 +63802,7 @@
         <v>1893</v>
       </c>
       <c r="H1176" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="I1176" t="s">
         <v>1995</v>
@@ -63820,7 +63820,7 @@
         <v>2018</v>
       </c>
       <c r="N1176" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O1176" t="s">
         <v>2031</v>
@@ -63943,7 +63943,7 @@
         <v>1893</v>
       </c>
       <c r="H1179" t="s">
-        <v>1955</v>
+        <v>1954</v>
       </c>
       <c r="I1179" t="s">
         <v>1995</v>
@@ -63961,7 +63961,7 @@
         <v>2018</v>
       </c>
       <c r="N1179" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O1179" t="s">
         <v>2031</v>
@@ -64122,7 +64122,7 @@
         <v>1893</v>
       </c>
       <c r="H1183" t="s">
-        <v>1949</v>
+        <v>1948</v>
       </c>
       <c r="I1183" t="s">
         <v>1989</v>
@@ -64172,7 +64172,7 @@
         <v>1893</v>
       </c>
       <c r="H1184" t="s">
-        <v>1949</v>
+        <v>1948</v>
       </c>
       <c r="I1184" t="s">
         <v>1989</v>
@@ -64222,7 +64222,7 @@
         <v>1893</v>
       </c>
       <c r="H1185" t="s">
-        <v>1949</v>
+        <v>1948</v>
       </c>
       <c r="I1185" t="s">
         <v>1989</v>
@@ -64272,7 +64272,7 @@
         <v>1893</v>
       </c>
       <c r="H1186" t="s">
-        <v>1949</v>
+        <v>1948</v>
       </c>
       <c r="I1186" t="s">
         <v>1989</v>
@@ -64571,7 +64571,7 @@
         <v>1893</v>
       </c>
       <c r="H1193" t="s">
-        <v>1952</v>
+        <v>1951</v>
       </c>
       <c r="I1193" t="s">
         <v>1995</v>
@@ -64589,7 +64589,7 @@
         <v>2018</v>
       </c>
       <c r="N1193" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O1193" t="s">
         <v>2029</v>
@@ -64621,7 +64621,7 @@
         <v>1893</v>
       </c>
       <c r="H1194" t="s">
-        <v>1949</v>
+        <v>1948</v>
       </c>
       <c r="I1194" t="s">
         <v>1989</v>
@@ -64780,7 +64780,7 @@
         <v>2018</v>
       </c>
       <c r="N1197" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O1197" t="s">
         <v>2029</v>
@@ -64871,7 +64871,7 @@
         <v>2018</v>
       </c>
       <c r="N1199" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O1199" t="s">
         <v>2031</v>
@@ -65100,7 +65100,7 @@
         <v>2016</v>
       </c>
       <c r="N1204" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O1204" t="s">
         <v>2029</v>
@@ -65214,7 +65214,7 @@
         <v>1893</v>
       </c>
       <c r="H1207" t="s">
-        <v>1956</v>
+        <v>1955</v>
       </c>
       <c r="I1207" t="s">
         <v>1995</v>
@@ -65232,7 +65232,7 @@
         <v>2018</v>
       </c>
       <c r="N1207" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O1207" t="s">
         <v>2029</v>
@@ -66115,7 +66115,7 @@
         <v>2016</v>
       </c>
       <c r="N1227" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O1227" t="s">
         <v>2029</v>
@@ -66320,7 +66320,7 @@
         <v>1893</v>
       </c>
       <c r="H1232" t="s">
-        <v>1952</v>
+        <v>1951</v>
       </c>
       <c r="I1232" t="s">
         <v>1995</v>
@@ -66338,7 +66338,7 @@
         <v>2017</v>
       </c>
       <c r="N1232" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O1232" t="s">
         <v>2029</v>
@@ -66764,7 +66764,7 @@
         <v>2017</v>
       </c>
       <c r="N1241" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O1241" t="s">
         <v>2031</v>
@@ -66987,7 +66987,7 @@
         <v>1893</v>
       </c>
       <c r="H1246" t="s">
-        <v>1949</v>
+        <v>1948</v>
       </c>
       <c r="I1246" t="s">
         <v>1989</v>
@@ -67528,7 +67528,7 @@
         <v>1893</v>
       </c>
       <c r="H1257" t="s">
-        <v>1952</v>
+        <v>1951</v>
       </c>
       <c r="I1257" t="s">
         <v>1995</v>
@@ -67546,7 +67546,7 @@
         <v>2016</v>
       </c>
       <c r="N1257" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O1257" t="s">
         <v>2031</v>
@@ -67872,7 +67872,7 @@
         <v>1893</v>
       </c>
       <c r="H1264" t="s">
-        <v>1954</v>
+        <v>1953</v>
       </c>
       <c r="I1264" t="s">
         <v>1995</v>
@@ -67890,7 +67890,7 @@
         <v>2018</v>
       </c>
       <c r="N1264" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O1264" t="s">
         <v>2031</v>
@@ -67922,7 +67922,7 @@
         <v>1893</v>
       </c>
       <c r="H1265" t="s">
-        <v>1954</v>
+        <v>1953</v>
       </c>
       <c r="I1265" t="s">
         <v>1995</v>
@@ -67940,7 +67940,7 @@
         <v>2018</v>
       </c>
       <c r="N1265" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O1265" t="s">
         <v>2031</v>
@@ -68069,7 +68069,7 @@
         <v>1893</v>
       </c>
       <c r="H1268" t="s">
-        <v>1949</v>
+        <v>1948</v>
       </c>
       <c r="I1268" t="s">
         <v>1989</v>
@@ -68439,7 +68439,7 @@
         <v>1893</v>
       </c>
       <c r="H1276" t="s">
-        <v>1952</v>
+        <v>1951</v>
       </c>
       <c r="I1276" t="s">
         <v>1995</v>
@@ -68457,7 +68457,7 @@
         <v>2018</v>
       </c>
       <c r="N1276" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O1276" t="s">
         <v>2029</v>
@@ -68627,7 +68627,7 @@
         <v>1893</v>
       </c>
       <c r="H1280" t="s">
-        <v>1954</v>
+        <v>1953</v>
       </c>
       <c r="I1280" t="s">
         <v>1995</v>
@@ -68645,7 +68645,7 @@
         <v>2017</v>
       </c>
       <c r="N1280" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O1280" t="s">
         <v>2031</v>
@@ -68795,7 +68795,7 @@
         <v>2018</v>
       </c>
       <c r="N1283" t="s">
-        <v>1945</v>
+        <v>1944</v>
       </c>
       <c r="O1283" t="s">
         <v>2029</v>
@@ -68827,7 +68827,7 @@
         <v>1893</v>
       </c>
       <c r="H1284" t="s">
-        <v>1949</v>
+        <v>1948</v>
       </c>
       <c r="I1284" t="s">
         <v>1989</v>

</xml_diff>

<commit_message>
Atualização automática: 2026-08-10 15:39
</commit_message>
<xml_diff>
--- a/data/base_formatada/Base.xlsx
+++ b/data/base_formatada/Base.xlsx
@@ -61120,7 +61120,7 @@
         <v>1893</v>
       </c>
       <c r="H1119" t="s">
-        <v>1896</v>
+        <v>1971</v>
       </c>
       <c r="I1119" t="s">
         <v>1989</v>
@@ -61170,7 +61170,7 @@
         <v>1893</v>
       </c>
       <c r="H1120" t="s">
-        <v>1896</v>
+        <v>1971</v>
       </c>
       <c r="I1120" t="s">
         <v>1989</v>
@@ -61220,7 +61220,7 @@
         <v>1893</v>
       </c>
       <c r="H1121" t="s">
-        <v>1896</v>
+        <v>1971</v>
       </c>
       <c r="I1121" t="s">
         <v>1989</v>

</xml_diff>

<commit_message>
Atualização automática: 2026-08-11 11:03
</commit_message>
<xml_diff>
--- a/data/base_formatada/Base.xlsx
+++ b/data/base_formatada/Base.xlsx
@@ -5671,7 +5671,7 @@
     <t>Cesar Ferreira</t>
   </si>
   <si>
-    <t>Claudio Correa</t>
+    <t>Lopes Assenço</t>
   </si>
   <si>
     <t>Edimir Santos</t>
@@ -55706,7 +55706,7 @@
         <v>1313</v>
       </c>
       <c r="E1007" t="s">
-        <v>1886</v>
+        <v>1885</v>
       </c>
       <c r="F1007" t="s">
         <v>1889</v>
@@ -59991,7 +59991,7 @@
         <v>1313</v>
       </c>
       <c r="E1096" t="s">
-        <v>1886</v>
+        <v>1885</v>
       </c>
       <c r="F1096" t="s">
         <v>1889</v>
@@ -64072,7 +64072,7 @@
         <v>1313</v>
       </c>
       <c r="E1182" t="s">
-        <v>1886</v>
+        <v>1885</v>
       </c>
       <c r="F1182" t="s">
         <v>1889</v>
@@ -65548,7 +65548,7 @@
         <v>1313</v>
       </c>
       <c r="E1215" t="s">
-        <v>1886</v>
+        <v>1885</v>
       </c>
       <c r="F1215" t="s">
         <v>1889</v>
@@ -66543,7 +66543,7 @@
         <v>1313</v>
       </c>
       <c r="E1237" t="s">
-        <v>1886</v>
+        <v>1885</v>
       </c>
       <c r="F1237" t="s">
         <v>1887</v>
@@ -67075,7 +67075,7 @@
         <v>1313</v>
       </c>
       <c r="E1248" t="s">
-        <v>1886</v>
+        <v>1885</v>
       </c>
       <c r="F1248" t="s">
         <v>1887</v>
@@ -68298,7 +68298,7 @@
         <v>1313</v>
       </c>
       <c r="E1273" t="s">
-        <v>1886</v>
+        <v>1885</v>
       </c>
       <c r="F1273" t="s">
         <v>1889</v>
@@ -68718,7 +68718,7 @@
         <v>1313</v>
       </c>
       <c r="E1282" t="s">
-        <v>1886</v>
+        <v>1885</v>
       </c>
       <c r="F1282" t="s">
         <v>1887</v>

</xml_diff>